<commit_message>
Fix format of CRC-cards
</commit_message>
<xml_diff>
--- a/docs/crc.xlsx
+++ b/docs/crc.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,8 +28,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,8 +45,13 @@
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -50,17 +59,88 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="007F8C8D"/>
+      </left>
+      <right style="thin">
+        <color rgb="007F8C8D"/>
+      </right>
+      <top style="thin">
+        <color rgb="007F8C8D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="007F8C8D"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="007F8C8D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="007F8C8D"/>
+      </right>
+      <top style="thin">
+        <color rgb="007F8C8D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="007F8C8D"/>
+      </right>
+      <top style="thin">
+        <color rgb="007F8C8D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="007F8C8D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="007F8C8D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="007F8C8D"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,151 +507,300 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="74" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Відповідальності</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Співпрацівники</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Зберігати ідентифікатор та ім'я працівника.</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>PayrollSheet, PayrollCalculation, Receipt</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Обов'язки класу</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>З ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>1. Зберігати ідентифікатор
+2. Зберігати повне ім’я
+3. Надавати ідентифікатор</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PayrollSheet
+PayrollCalculation
+Receipt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1"/>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>DirectorOrder</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Підтверджувати чинність наказу та дозволяти його відкликання.</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Обов'язки класу</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>З ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>1. Зберігати ідентифікатор
+2. Перевіряти чинність
+3. Відкликати наказ</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>PayrollSheet</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="8" ht="48" customHeight="1"/>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>PayrollSheet</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Керувати складом відомості, перевіряти передумови та створювати нарахування.</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>DirectorOrder, Employee, PayrollRule, PayrollCalculation</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Обов'язки класу</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>З ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="64" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>1. Керувати складом працівників
+2. Перевіряти передумови
+3. Створювати нарахування
+4. Знаходити нарахування</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>DirectorOrder
+Employee
+PayrollRule
+PayrollCalculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1"/>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>PayrollCalculation</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Зберігати результат нарахування конкретного працівника.</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Employee, PayrollSheet, Receipt</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Обов'язки класу</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>З ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>1. Зберігати працівника
+2. Зберігати суму нарахування</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Employee
+PayrollSheet
+Receipt</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1"/>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Receipt</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Подавати працівникові його завершене нарахування.</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Employee, PayrollCalculation</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Обов'язки класу</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>З ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>1. Подавати завершене нарахування</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Employee
+PayrollCalculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>BasePayrollRule</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Надавати спільну абстрактну основу правила нарахування та контракт PayrollRule.</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>PayrollRule, StandardPayrollRule</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Обов'язки класу</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>З ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>1. Надавати основу правила
+2. Визначати контракт правила</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>PayrollRule
+StandardPayrollRule</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1"/>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>StandardPayrollRule</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Обчислювати суму за стандартним правилом і реалізовувати PayrollRule.</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>BasePayrollRule, Employee, PayrollSheet</t>
-        </is>
-      </c>
-    </row>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Обов'язки класу</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>З ким співпрацює</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>1. Обчислювати суму нарахування</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>BasePayrollRule
+Employee
+PayrollSheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1"/>
+    <row r="29" ht="32" customHeight="1"/>
+    <row r="31" ht="24" customHeight="1"/>
+    <row r="32" ht="22" customHeight="1"/>
+    <row r="33" ht="22" customHeight="1"/>
+    <row r="34" ht="48" customHeight="1"/>
   </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A10:B10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>